<commit_message>
Refine NGTG drop-reason buckets by reading both remarks columns
</commit_message>
<xml_diff>
--- a/NGTG_Drop_Reasons_Feb_March.xlsx
+++ b/NGTG_Drop_Reasons_Feb_March.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +32,11 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +51,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,13 +85,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -455,10 +467,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
@@ -483,102 +495,102 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generic - no specific reason given</t>
+          <t>Low product count / SKUs</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>101</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Low product count / SKUs</t>
+          <t>Products/stock not ready (start later / pause)</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Products/stock not ready (start later)</t>
+          <t>Refund request</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Refund request</t>
+          <t>Out of criteria (category / product type / dimension)</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Out of criteria (category/product type)</t>
+          <t>No contact / RNR / not responding</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>No contact / RNR / not responding</t>
+          <t>No GST / license / registration</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>7</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Duplicate / old / mistaken lead</t>
+          <t>Pricing / AOV / commission / COGS</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Pricing / AOV / commission / COGS</t>
+          <t>Duplicate / old / mistaken / churned account</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>9</v>
@@ -587,24 +599,24 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>No GST / license</t>
+          <t>Sales POC issue / mis-sold / service delay</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Personal / out of country</t>
+          <t>Personal / out of country / global issues</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>4</v>
@@ -613,14 +625,14 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>No marketing budget / financial</t>
+          <t>Expectation mismatch / high expectations</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -639,7 +651,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Sales POC issue / mis-sold</t>
+          <t>No marketing budget / financial</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -650,15 +662,54 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chose competitor / another platform</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Generic vague ("don't want to continue")</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>No reason logged (blank remarks)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Total churned</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B18" s="7" t="n">
         <v>219</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C18" s="7" t="n">
         <v>288</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Disposition Share tab (Feb vs March) alongside drop-reason buckets
</commit_message>
<xml_diff>
--- a/NGTG_Drop_Reasons_Feb_March.xlsx
+++ b/NGTG_Drop_Reasons_Feb_March.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Drop Reasons" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Disposition Share" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Drop Reason Buckets" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -85,21 +86,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -467,6 +471,107 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Disposition reason</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>asked_to_drop_the_lead</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>seller_wants_to_drop_out</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>not_in_shopdeck_criteria</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>photoshoot_not_available</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Total churned</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>219</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>288</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -498,10 +603,10 @@
           <t>Low product count / SKUs</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="6" t="n">
         <v>48</v>
       </c>
     </row>
@@ -511,10 +616,10 @@
           <t>Products/stock not ready (start later / pause)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="6" t="n">
         <v>38</v>
       </c>
     </row>
@@ -524,10 +629,10 @@
           <t>Refund request</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="6" t="n">
         <v>31</v>
       </c>
     </row>
@@ -537,10 +642,10 @@
           <t>Out of criteria (category / product type / dimension)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -550,10 +655,10 @@
           <t>No contact / RNR / not responding</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -563,10 +668,10 @@
           <t>No GST / license / registration</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -576,10 +681,10 @@
           <t>Pricing / AOV / commission / COGS</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="6" t="n">
         <v>8</v>
       </c>
     </row>
@@ -589,10 +694,10 @@
           <t>Duplicate / old / mistaken / churned account</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="6" t="n">
         <v>9</v>
       </c>
     </row>
@@ -602,10 +707,10 @@
           <t>Sales POC issue / mis-sold / service delay</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -615,10 +720,10 @@
           <t>Personal / out of country / global issues</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -628,88 +733,88 @@
           <t>Expectation mismatch / high expectations</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Inventory mgmt / no website need</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>3</v>
+          <t>Chose competitor / another platform</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>No marketing budget / financial</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>2</v>
+          <t>Inventory mgmt / no website need</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Chose competitor / another platform</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
+          <t>No marketing budget / financial</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="3" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Generic vague ("don't want to continue")</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="8" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>No reason logged (blank remarks)</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="8" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Total churned</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="5" t="n">
         <v>219</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="5" t="n">
         <v>288</v>
       </c>
     </row>

</xml_diff>